<commit_message>
First push for the "Data" sheet validation.
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_ErrorSample.xlsx
+++ b/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_ErrorSample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20415"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2AF0D4-4E51-4157-885C-4C3D1A28B61F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EC9501-D02B-4B81-BF47-0AADA4EC1564}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13425" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -430,9 +430,6 @@
     <t>https://doi.org/10.1016/j.apenergy.2019.113632</t>
   </si>
   <si>
-    <t>diesel-powered bus</t>
-  </si>
-  <si>
     <t>battery electric bus</t>
   </si>
   <si>
@@ -641,6 +638,9 @@
   </si>
   <si>
     <t>TEST</t>
+  </si>
+  <si>
+    <t>bus</t>
   </si>
 </sst>
 </file>
@@ -1131,21 +1131,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="15" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1172,6 +1157,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1530,18 +1530,18 @@
       <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="74"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="69"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="72" t="s">
+      <c r="F2" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="74"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="69"/>
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11">
@@ -1559,7 +1559,7 @@
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="75" t="s">
+      <c r="B4" s="70" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="10" t="s">
@@ -1569,7 +1569,7 @@
         <v>28</v>
       </c>
       <c r="E4" s="51" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F4" s="43" t="s">
         <v>30</v>
@@ -1583,7 +1583,7 @@
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="76"/>
+      <c r="B5" s="71"/>
       <c r="C5" s="14" t="s">
         <v>31</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>126</v>
       </c>
       <c r="E5" s="51" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F5" s="52" t="s">
         <v>29</v>
@@ -1611,7 +1611,7 @@
         <v>21</v>
       </c>
       <c r="E6" s="51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F6" s="44" t="s">
         <v>0</v>
@@ -1627,7 +1627,7 @@
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" s="77" t="s">
+      <c r="B7" s="72" t="s">
         <v>34</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -1637,7 +1637,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="51" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F7" s="44" t="s">
         <v>1</v>
@@ -1646,7 +1646,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I7" s="20"/>
       <c r="J7" s="1" t="s">
@@ -1658,7 +1658,7 @@
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8" s="77"/>
+      <c r="B8" s="72"/>
       <c r="C8" s="14" t="s">
         <v>36</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>3</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F8" s="44" t="s">
         <v>6</v>
@@ -1682,7 +1682,7 @@
       <c r="A9">
         <v>6</v>
       </c>
-      <c r="B9" s="77"/>
+      <c r="B9" s="72"/>
       <c r="C9" s="14" t="s">
         <v>37</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>108</v>
       </c>
       <c r="E9" s="51" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F9" s="44" t="s">
         <v>7</v>
@@ -1706,7 +1706,7 @@
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="B10" s="77"/>
+      <c r="B10" s="72"/>
       <c r="C10" s="14" t="s">
         <v>38</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>108</v>
       </c>
       <c r="E10" s="51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F10" s="46" t="s">
         <v>2</v>
@@ -1723,7 +1723,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I10" s="36">
         <v>20</v>
@@ -1734,7 +1734,7 @@
       <c r="A11">
         <v>8</v>
       </c>
-      <c r="B11" s="78" t="s">
+      <c r="B11" s="73" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="33" t="s">
@@ -1744,13 +1744,13 @@
         <v>109</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H11" s="48" t="s">
         <v>8</v>
@@ -1767,7 +1767,7 @@
       <c r="A12">
         <v>9</v>
       </c>
-      <c r="B12" s="79"/>
+      <c r="B12" s="74"/>
       <c r="C12" s="33" t="s">
         <v>41</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>117</v>
       </c>
       <c r="E12" s="51" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F12" s="25" t="s">
         <v>14</v>
@@ -1787,7 +1787,7 @@
         <v>16</v>
       </c>
       <c r="I12" s="66" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>29</v>
@@ -1798,7 +1798,7 @@
       <c r="A13">
         <v>10</v>
       </c>
-      <c r="B13" s="79"/>
+      <c r="B13" s="74"/>
       <c r="C13" s="33" t="s">
         <v>115</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>120</v>
       </c>
       <c r="E13" s="51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F13" s="25" t="s">
         <v>11</v>
@@ -1818,7 +1818,7 @@
         <v>17</v>
       </c>
       <c r="I13" s="66" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>29</v>
@@ -1829,7 +1829,7 @@
       <c r="A14">
         <v>11</v>
       </c>
-      <c r="B14" s="79"/>
+      <c r="B14" s="74"/>
       <c r="C14" s="33" t="s">
         <v>42</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>129</v>
       </c>
       <c r="E14" s="51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F14" s="26" t="s">
         <v>15</v>
@@ -1849,7 +1849,7 @@
         <v>18</v>
       </c>
       <c r="I14" s="66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>29</v>
@@ -1860,7 +1860,7 @@
       <c r="A15">
         <v>12</v>
       </c>
-      <c r="B15" s="79"/>
+      <c r="B15" s="74"/>
       <c r="C15" s="33" t="s">
         <v>43</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>21</v>
       </c>
       <c r="E15" s="51" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F15" s="25" t="s">
         <v>12</v>
@@ -1880,7 +1880,7 @@
         <v>19</v>
       </c>
       <c r="I15" s="66" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>29</v>
@@ -1891,7 +1891,7 @@
       <c r="A16">
         <v>13</v>
       </c>
-      <c r="B16" s="79"/>
+      <c r="B16" s="74"/>
       <c r="C16" s="33" t="s">
         <v>44</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>21</v>
       </c>
       <c r="E16" s="51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F16" s="52" t="s">
         <v>29</v>
@@ -1909,7 +1909,7 @@
         <v>20</v>
       </c>
       <c r="I16" s="66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>29</v>
@@ -1920,7 +1920,7 @@
       <c r="A17">
         <v>14</v>
       </c>
-      <c r="B17" s="79"/>
+      <c r="B17" s="74"/>
       <c r="C17" s="33" t="s">
         <v>45</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>119</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F17" s="52" t="s">
         <v>29</v>
@@ -1941,7 +1941,7 @@
       <c r="A18">
         <v>15</v>
       </c>
-      <c r="B18" s="79"/>
+      <c r="B18" s="74"/>
       <c r="C18" s="33" t="s">
         <v>46</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>130</v>
       </c>
       <c r="E18" s="51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F18" s="52" t="s">
         <v>29</v>
@@ -1961,7 +1961,7 @@
       <c r="A19">
         <v>16</v>
       </c>
-      <c r="B19" s="79"/>
+      <c r="B19" s="74"/>
       <c r="C19" s="33" t="s">
         <v>47</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>125</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F19" s="52" t="s">
         <v>29</v>
@@ -1981,7 +1981,7 @@
       <c r="A20">
         <v>17</v>
       </c>
-      <c r="B20" s="79"/>
+      <c r="B20" s="74"/>
       <c r="C20" s="33" t="s">
         <v>48</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>110</v>
       </c>
       <c r="E20" s="51" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F20" s="52" t="s">
         <v>29</v>
@@ -2001,7 +2001,7 @@
       <c r="A21">
         <v>18</v>
       </c>
-      <c r="B21" s="80" t="s">
+      <c r="B21" s="75" t="s">
         <v>49</v>
       </c>
       <c r="C21" s="33" t="s">
@@ -2011,7 +2011,7 @@
         <v>127</v>
       </c>
       <c r="E21" s="51" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F21" s="53" t="s">
         <v>29</v>
@@ -2025,7 +2025,7 @@
       <c r="A22">
         <v>19</v>
       </c>
-      <c r="B22" s="80"/>
+      <c r="B22" s="75"/>
       <c r="C22" s="33" t="s">
         <v>51</v>
       </c>
@@ -2033,7 +2033,7 @@
         <v>121</v>
       </c>
       <c r="E22" s="51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F22" s="62" t="s">
         <v>29</v>
@@ -2044,7 +2044,7 @@
       <c r="A23">
         <v>20</v>
       </c>
-      <c r="B23" s="80"/>
+      <c r="B23" s="75"/>
       <c r="C23" s="33" t="s">
         <v>52</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>122</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F23" s="62" t="s">
         <v>29</v>
@@ -2063,7 +2063,7 @@
       <c r="A24">
         <v>21</v>
       </c>
-      <c r="B24" s="80"/>
+      <c r="B24" s="75"/>
       <c r="C24" s="33" t="s">
         <v>53</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F24" s="62" t="s">
         <v>29</v>
@@ -2083,7 +2083,7 @@
       <c r="A25">
         <v>22</v>
       </c>
-      <c r="B25" s="80"/>
+      <c r="B25" s="75"/>
       <c r="C25" s="33" t="s">
         <v>20</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>21</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F25" s="62" t="s">
         <v>29</v>
@@ -2103,7 +2103,7 @@
       <c r="A26">
         <v>23</v>
       </c>
-      <c r="B26" s="67" t="s">
+      <c r="B26" s="76" t="s">
         <v>54</v>
       </c>
       <c r="C26" s="41" t="s">
@@ -2113,7 +2113,7 @@
         <v>14</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F26" s="62" t="s">
         <v>29</v>
@@ -2126,7 +2126,7 @@
       <c r="A27">
         <v>24</v>
       </c>
-      <c r="B27" s="67"/>
+      <c r="B27" s="76"/>
       <c r="C27" s="41" t="s">
         <v>56</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>7</v>
       </c>
       <c r="E27" s="51" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F27" s="62" t="s">
         <v>29</v>
@@ -2146,7 +2146,7 @@
       <c r="A28">
         <v>25</v>
       </c>
-      <c r="B28" s="67"/>
+      <c r="B28" s="76"/>
       <c r="C28" s="41" t="s">
         <v>57</v>
       </c>
@@ -2166,7 +2166,7 @@
       <c r="A29">
         <v>26</v>
       </c>
-      <c r="B29" s="67"/>
+      <c r="B29" s="76"/>
       <c r="C29" s="41" t="s">
         <v>58</v>
       </c>
@@ -2186,7 +2186,7 @@
       <c r="A30">
         <v>27</v>
       </c>
-      <c r="B30" s="67"/>
+      <c r="B30" s="76"/>
       <c r="C30" s="41" t="s">
         <v>59</v>
       </c>
@@ -2206,7 +2206,7 @@
       <c r="A31">
         <v>28</v>
       </c>
-      <c r="B31" s="67"/>
+      <c r="B31" s="76"/>
       <c r="C31" s="41" t="s">
         <v>60</v>
       </c>
@@ -2226,7 +2226,7 @@
       <c r="A32">
         <v>29</v>
       </c>
-      <c r="B32" s="67"/>
+      <c r="B32" s="76"/>
       <c r="C32" s="41" t="s">
         <v>61</v>
       </c>
@@ -2245,7 +2245,7 @@
       <c r="A33">
         <v>30</v>
       </c>
-      <c r="B33" s="67"/>
+      <c r="B33" s="76"/>
       <c r="C33" s="41" t="s">
         <v>62</v>
       </c>
@@ -2264,7 +2264,7 @@
       <c r="A34">
         <v>31</v>
       </c>
-      <c r="B34" s="67"/>
+      <c r="B34" s="76"/>
       <c r="C34" s="41" t="s">
         <v>63</v>
       </c>
@@ -2283,7 +2283,7 @@
       <c r="A35">
         <v>32</v>
       </c>
-      <c r="B35" s="67"/>
+      <c r="B35" s="76"/>
       <c r="C35" s="31" t="s">
         <v>64</v>
       </c>
@@ -2303,7 +2303,7 @@
       <c r="A36">
         <v>33</v>
       </c>
-      <c r="B36" s="67"/>
+      <c r="B36" s="76"/>
       <c r="C36" s="31" t="s">
         <v>65</v>
       </c>
@@ -2323,7 +2323,7 @@
       <c r="A37">
         <v>34</v>
       </c>
-      <c r="B37" s="67"/>
+      <c r="B37" s="76"/>
       <c r="C37" s="31" t="s">
         <v>66</v>
       </c>
@@ -2342,7 +2342,7 @@
       <c r="A38">
         <v>35</v>
       </c>
-      <c r="B38" s="67"/>
+      <c r="B38" s="76"/>
       <c r="C38" s="31" t="s">
         <v>67</v>
       </c>
@@ -2362,7 +2362,7 @@
       <c r="A39">
         <v>36</v>
       </c>
-      <c r="B39" s="67"/>
+      <c r="B39" s="76"/>
       <c r="C39" s="31" t="s">
         <v>68</v>
       </c>
@@ -2383,7 +2383,7 @@
       <c r="A40">
         <v>37</v>
       </c>
-      <c r="B40" s="67"/>
+      <c r="B40" s="76"/>
       <c r="C40" s="31" t="s">
         <v>69</v>
       </c>
@@ -2405,7 +2405,7 @@
       <c r="A41">
         <v>38</v>
       </c>
-      <c r="B41" s="67"/>
+      <c r="B41" s="76"/>
       <c r="C41" s="31" t="s">
         <v>70</v>
       </c>
@@ -2426,7 +2426,7 @@
       <c r="A42">
         <v>39</v>
       </c>
-      <c r="B42" s="67"/>
+      <c r="B42" s="76"/>
       <c r="C42" s="31" t="s">
         <v>71</v>
       </c>
@@ -2447,7 +2447,7 @@
       <c r="A43">
         <v>40</v>
       </c>
-      <c r="B43" s="67"/>
+      <c r="B43" s="76"/>
       <c r="C43" s="31" t="s">
         <v>72</v>
       </c>
@@ -2469,7 +2469,7 @@
       <c r="A44">
         <v>41</v>
       </c>
-      <c r="B44" s="67"/>
+      <c r="B44" s="76"/>
       <c r="C44" s="31" t="s">
         <v>73</v>
       </c>
@@ -2491,7 +2491,7 @@
       <c r="A45">
         <v>42</v>
       </c>
-      <c r="B45" s="67"/>
+      <c r="B45" s="76"/>
       <c r="C45" s="31" t="s">
         <v>74</v>
       </c>
@@ -2515,7 +2515,7 @@
       <c r="A46">
         <v>43</v>
       </c>
-      <c r="B46" s="67"/>
+      <c r="B46" s="76"/>
       <c r="C46" s="31" t="s">
         <v>75</v>
       </c>
@@ -2538,7 +2538,7 @@
       <c r="A47">
         <v>44</v>
       </c>
-      <c r="B47" s="67"/>
+      <c r="B47" s="76"/>
       <c r="C47" s="31" t="s">
         <v>76</v>
       </c>
@@ -2559,7 +2559,7 @@
       <c r="A48">
         <v>45</v>
       </c>
-      <c r="B48" s="67"/>
+      <c r="B48" s="76"/>
       <c r="C48" s="31" t="s">
         <v>77</v>
       </c>
@@ -2580,7 +2580,7 @@
       <c r="A49">
         <v>46</v>
       </c>
-      <c r="B49" s="67"/>
+      <c r="B49" s="76"/>
       <c r="C49" s="31" t="s">
         <v>78</v>
       </c>
@@ -2603,7 +2603,7 @@
       <c r="A50">
         <v>47</v>
       </c>
-      <c r="B50" s="67"/>
+      <c r="B50" s="76"/>
       <c r="C50" s="23" t="s">
         <v>79</v>
       </c>
@@ -2611,7 +2611,7 @@
         <v>111</v>
       </c>
       <c r="E50" s="51" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F50" s="62" t="s">
         <v>29</v>
@@ -2625,7 +2625,7 @@
       <c r="A51">
         <v>48</v>
       </c>
-      <c r="B51" s="67"/>
+      <c r="B51" s="76"/>
       <c r="C51" s="23" t="s">
         <v>80</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>124</v>
       </c>
       <c r="E51" s="51" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F51" s="62" t="s">
         <v>29</v>
@@ -2646,7 +2646,7 @@
       <c r="A52">
         <v>49</v>
       </c>
-      <c r="B52" s="67"/>
+      <c r="B52" s="76"/>
       <c r="C52" s="23" t="s">
         <v>81</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>112</v>
       </c>
       <c r="E52" s="51" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F52" s="62" t="s">
         <v>29</v>
@@ -2668,7 +2668,7 @@
       <c r="A53">
         <v>50</v>
       </c>
-      <c r="B53" s="68" t="s">
+      <c r="B53" s="77" t="s">
         <v>82</v>
       </c>
       <c r="C53" s="14" t="s">
@@ -2678,7 +2678,7 @@
         <v>84</v>
       </c>
       <c r="E53" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F53" s="62" t="s">
         <v>29</v>
@@ -2690,7 +2690,7 @@
       <c r="A54">
         <v>51</v>
       </c>
-      <c r="B54" s="68"/>
+      <c r="B54" s="77"/>
       <c r="C54" s="14" t="s">
         <v>85</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>86</v>
       </c>
       <c r="E54" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F54" s="62" t="s">
         <v>29</v>
@@ -2710,7 +2710,7 @@
       <c r="A55">
         <v>52</v>
       </c>
-      <c r="B55" s="68"/>
+      <c r="B55" s="77"/>
       <c r="C55" s="14" t="s">
         <v>87</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>123</v>
       </c>
       <c r="E55" s="51" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F55" s="62" t="s">
         <v>29</v>
@@ -2730,7 +2730,7 @@
       <c r="A56">
         <v>53</v>
       </c>
-      <c r="B56" s="68"/>
+      <c r="B56" s="77"/>
       <c r="C56" s="14" t="s">
         <v>88</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>131</v>
       </c>
       <c r="E56" s="51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F56" s="62" t="s">
         <v>29</v>
@@ -2750,7 +2750,7 @@
       <c r="A57">
         <v>54</v>
       </c>
-      <c r="B57" s="68"/>
+      <c r="B57" s="77"/>
       <c r="C57" s="23" t="s">
         <v>89</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>113</v>
       </c>
       <c r="E57" s="51" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F57" s="62" t="s">
         <v>29</v>
@@ -2770,13 +2770,13 @@
       <c r="A58">
         <v>55</v>
       </c>
-      <c r="B58" s="68"/>
+      <c r="B58" s="77"/>
       <c r="C58" s="14" t="s">
         <v>90</v>
       </c>
       <c r="D58" s="54"/>
       <c r="E58" s="51" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F58" s="62" t="s">
         <v>29</v>
@@ -2788,7 +2788,7 @@
       <c r="A59">
         <v>56</v>
       </c>
-      <c r="B59" s="68"/>
+      <c r="B59" s="77"/>
       <c r="C59" s="14" t="s">
         <v>91</v>
       </c>
@@ -2796,7 +2796,7 @@
         <v>131</v>
       </c>
       <c r="E59" s="51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F59" s="62" t="s">
         <v>29</v>
@@ -2811,7 +2811,7 @@
       <c r="A60">
         <v>57</v>
       </c>
-      <c r="B60" s="68"/>
+      <c r="B60" s="77"/>
       <c r="C60" s="14" t="s">
         <v>92</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>1</v>
       </c>
       <c r="E60" s="51" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F60" s="62" t="s">
         <v>29</v>
@@ -2834,7 +2834,7 @@
       <c r="A61">
         <v>58</v>
       </c>
-      <c r="B61" s="69" t="s">
+      <c r="B61" s="78" t="s">
         <v>93</v>
       </c>
       <c r="C61" s="14" t="s">
@@ -2844,7 +2844,7 @@
         <v>45400</v>
       </c>
       <c r="E61" s="51" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F61" s="62" t="s">
         <v>29</v>
@@ -2857,7 +2857,7 @@
       <c r="A62">
         <v>59</v>
       </c>
-      <c r="B62" s="69"/>
+      <c r="B62" s="78"/>
       <c r="C62" s="14" t="s">
         <v>95</v>
       </c>
@@ -2865,7 +2865,7 @@
         <v>45400</v>
       </c>
       <c r="E62" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F62" s="62" t="s">
         <v>29</v>
@@ -2878,7 +2878,7 @@
       <c r="A63">
         <v>60</v>
       </c>
-      <c r="B63" s="69"/>
+      <c r="B63" s="78"/>
       <c r="C63" s="14" t="s">
         <v>96</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>114</v>
       </c>
       <c r="E63" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F63" s="62" t="s">
         <v>29</v>
@@ -2900,7 +2900,7 @@
       <c r="A64">
         <v>61</v>
       </c>
-      <c r="B64" s="69"/>
+      <c r="B64" s="78"/>
       <c r="C64" s="14" t="s">
         <v>97</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>98</v>
       </c>
       <c r="E64" s="51" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F64" s="62" t="s">
         <v>29</v>
@@ -2922,7 +2922,7 @@
       <c r="A65">
         <v>62</v>
       </c>
-      <c r="B65" s="69"/>
+      <c r="B65" s="78"/>
       <c r="C65" s="14" t="s">
         <v>99</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>45455</v>
       </c>
       <c r="E65" s="51" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F65" s="62" t="s">
         <v>29</v>
@@ -2942,7 +2942,7 @@
       <c r="A66">
         <v>63</v>
       </c>
-      <c r="B66" s="69"/>
+      <c r="B66" s="78"/>
       <c r="C66" s="14" t="s">
         <v>100</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>128</v>
       </c>
       <c r="E66" s="51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F66" s="62" t="s">
         <v>29</v>
@@ -2961,13 +2961,13 @@
       <c r="A67">
         <v>64</v>
       </c>
-      <c r="B67" s="69"/>
+      <c r="B67" s="78"/>
       <c r="C67" s="14" t="s">
         <v>101</v>
       </c>
       <c r="D67" s="61"/>
       <c r="E67" s="51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F67" s="62" t="s">
         <v>29</v>
@@ -2978,7 +2978,7 @@
       <c r="A68">
         <v>65</v>
       </c>
-      <c r="B68" s="70" t="s">
+      <c r="B68" s="79" t="s">
         <v>102</v>
       </c>
       <c r="C68" s="33" t="s">
@@ -2996,7 +2996,7 @@
       <c r="A69">
         <v>66</v>
       </c>
-      <c r="B69" s="70"/>
+      <c r="B69" s="79"/>
       <c r="C69" s="33" t="s">
         <v>104</v>
       </c>
@@ -3012,7 +3012,7 @@
       <c r="A70">
         <v>67</v>
       </c>
-      <c r="B70" s="70"/>
+      <c r="B70" s="79"/>
       <c r="C70" s="33" t="s">
         <v>105</v>
       </c>
@@ -3026,7 +3026,7 @@
       <c r="A71">
         <v>68</v>
       </c>
-      <c r="B71" s="70"/>
+      <c r="B71" s="79"/>
       <c r="C71" s="33" t="s">
         <v>106</v>
       </c>
@@ -3040,7 +3040,7 @@
       <c r="A72">
         <v>69</v>
       </c>
-      <c r="B72" s="71"/>
+      <c r="B72" s="80"/>
       <c r="C72" s="34" t="s">
         <v>107</v>
       </c>
@@ -3052,16 +3052,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B26:B52"/>
+    <mergeCell ref="B53:B60"/>
+    <mergeCell ref="B61:B67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:I2"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="B11:B20"/>
     <mergeCell ref="B21:B25"/>
-    <mergeCell ref="B26:B52"/>
-    <mergeCell ref="B53:B60"/>
-    <mergeCell ref="B61:B67"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>
@@ -3098,7 +3098,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>12</v>
@@ -3119,15 +3119,15 @@
         <v>11</v>
       </c>
       <c r="J1" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K1" s="37" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="37" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="B2" s="37" t="s">
         <v>13</v>
@@ -3156,7 +3156,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>13</v>
@@ -3185,7 +3185,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B4" s="37" t="s">
         <v>13</v>
@@ -3214,7 +3214,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" s="37" t="s">
         <v>13</v>
@@ -3243,7 +3243,7 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B6" s="37" t="s">
         <v>13</v>
@@ -3272,7 +3272,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B7" s="37" t="s">
         <v>13</v>
@@ -3301,7 +3301,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="37" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B8" s="37" t="s">
         <v>13</v>
@@ -3330,7 +3330,7 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B9" s="37" t="s">
         <v>13</v>
@@ -3359,7 +3359,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B10" s="37" t="s">
         <v>13</v>
@@ -3388,7 +3388,7 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="37" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B11" s="37" t="s">
         <v>13</v>
@@ -3417,7 +3417,7 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B12" s="37" t="s">
         <v>13</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B13" s="37" t="s">
         <v>13</v>
@@ -3475,7 +3475,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B14" s="37" t="s">
         <v>13</v>
@@ -3504,7 +3504,7 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B15" s="37" t="s">
         <v>13</v>
@@ -3533,7 +3533,7 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B16" s="37" t="s">
         <v>13</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B17" s="37" t="s">
         <v>13</v>
@@ -3591,7 +3591,7 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B18" s="37" t="s">
         <v>13</v>
@@ -3620,7 +3620,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B19" s="37" t="s">
         <v>13</v>
@@ -3649,7 +3649,7 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B20" s="37" t="s">
         <v>13</v>
@@ -3678,7 +3678,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B21" s="37" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Levenshtein function was added for the close match search.
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_ErrorSample.xlsx
+++ b/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_ErrorSample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20416"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AC7786-C135-43BC-A30B-8E3BDBA9D3BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E5C054-0FFB-4B8B-8CEC-97F6C32C4865}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13425" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="203">
   <si>
     <t>Format_Version</t>
   </si>
@@ -638,6 +638,9 @@
   </si>
   <si>
     <t>bus</t>
+  </si>
+  <si>
+    <t>Chine</t>
   </si>
 </sst>
 </file>
@@ -3153,7 +3156,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>119</v>
+        <v>202</v>
       </c>
       <c r="D3" s="37" t="s">
         <v>125</v>

</xml_diff>